<commit_message>
3. Great Things happens at Night Only.
</commit_message>
<xml_diff>
--- a/raw_data/Book1.xlsx
+++ b/raw_data/Book1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Different Folder\Code\python\Scrapping the Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Different Folder\Code\python\Scrapping the Data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{197FBBB1-34D8-4AA6-A90A-8F36C8B19743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F28BC057-4E8D-4C2D-84C4-05F512CE6527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{43B1A38A-3033-4D74-9A5B-D8150D859200}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="9960" xr2:uid="{43B1A38A-3033-4D74-9A5B-D8150D859200}"/>
   </bookViews>
   <sheets>
     <sheet name="Book1" sheetId="1" r:id="rId1"/>
@@ -20,16 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Column1</t>
-  </si>
-  <si>
-    <t>Column2</t>
-  </si>
-  <si>
-    <t>Column3</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="33">
   <si>
     <t>T2</t>
   </si>
@@ -50,6 +41,84 @@
   </si>
   <si>
     <t>hey there 123</t>
+  </si>
+  <si>
+    <t>T4</t>
+  </si>
+  <si>
+    <t>Potter</t>
+  </si>
+  <si>
+    <t>David</t>
+  </si>
+  <si>
+    <t>Ram</t>
+  </si>
+  <si>
+    <t>Rohan</t>
+  </si>
+  <si>
+    <t>Econ</t>
+  </si>
+  <si>
+    <t>T5</t>
+  </si>
+  <si>
+    <t>T7</t>
+  </si>
+  <si>
+    <t>T8</t>
+  </si>
+  <si>
+    <t>T9</t>
+  </si>
+  <si>
+    <t>SWOIFNV</t>
+  </si>
+  <si>
+    <t>OPJHY</t>
+  </si>
+  <si>
+    <t>wefo</t>
+  </si>
+  <si>
+    <t>kcnsd496832</t>
+  </si>
+  <si>
+    <t>Salary</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Employee ID</t>
+  </si>
+  <si>
+    <t>Ext Data</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>Mangement</t>
+  </si>
+  <si>
+    <t>it</t>
+  </si>
+  <si>
+    <t>HR</t>
+  </si>
+  <si>
+    <t>EC</t>
+  </si>
+  <si>
+    <t>ec</t>
+  </si>
+  <si>
+    <t>mangement</t>
   </si>
 </sst>
 </file>
@@ -890,48 +959,137 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF7CBE47-948E-4BB6-A314-2175197FA50D}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
+      <c r="D2">
+        <v>5000</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
+      <c r="D3">
+        <v>6000</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
+      <c r="E4" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B4">
-        <v>123</v>
-      </c>
-      <c r="C4" t="s">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
         <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6">
+        <v>8000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>2700</v>
+      </c>
+      <c r="E7" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
+        <v>4500</v>
+      </c>
+      <c r="E8" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>